<commit_message>
balance: raise generator rates (T2×100, T3×10, T4-T7×3)
T2: 0.0005 → 0.05, T3: 0.0004 → 0.004, T4: 0.00032 → 0.00096,
T5: 0.000256 → 0.000768, T6: 0.000205 → 0.000615, T7: 0.000164 → 0.000492.

Sim (40 days): P1 day 6, P2 day 12.5, full 54/54 day 34.
CC/s: 12 → 7M (day 1) → 625T (day 12). Early game noticeably snappier.
⚠ Visa gate now weak at high CC/s — consider raising transit costs later.

Updated: xlsx, playthrough_log.csv, ECONOMY-BALANCE.md, game.html CONFIG.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/economy-model/galactic_bureaucracy_economy.xlsx
+++ b/design/economy-model/galactic_bureaucracy_economy.xlsx
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="E7" s="131" t="n">
-        <v>0.0005</v>
+        <v>0.05</v>
       </c>
       <c r="F7" s="105" t="n">
         <v>800</v>
@@ -2120,7 +2120,7 @@
         </is>
       </c>
       <c r="E8" s="130" t="n">
-        <v>0.0004</v>
+        <v>0.004</v>
       </c>
       <c r="F8" s="108" t="n">
         <v>60000</v>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="E9" s="131" t="n">
-        <v>0.00032</v>
+        <v>0.00096</v>
       </c>
       <c r="F9" s="105" t="n">
         <v>9000000</v>
@@ -2182,7 +2182,7 @@
         </is>
       </c>
       <c r="E10" s="130" t="n">
-        <v>0.000256</v>
+        <v>0.000768</v>
       </c>
       <c r="F10" s="108" t="n">
         <v>1600000000</v>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="E11" s="131" t="n">
-        <v>0.000205</v>
+        <v>0.000615</v>
       </c>
       <c r="F11" s="105" t="n">
         <v>320000000000</v>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="E12" s="130" t="n">
-        <v>0.000164</v>
+        <v>0.000492</v>
       </c>
       <c r="F12" s="108" t="n">
         <v>72000000000000</v>

</xml_diff>